<commit_message>
Made schema changes, proposed v3 of schema design, added cutoff details documents of 2024, 2025 (2023 link available)
</commit_message>
<xml_diff>
--- a/data/raw_data/mumbai_raw_data (empty).xlsx
+++ b/data/raw_data/mumbai_raw_data (empty).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Farheen\DSE-Compass\data\raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5F9FB6-29E7-448D-BD98-E61306C1F768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEB0BCB7-4679-4E9A-9219-9791DACC03D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="college_details" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="39">
   <si>
     <t>college_id</t>
   </si>
@@ -151,6 +151,9 @@
   </si>
   <si>
     <t>avg_package</t>
+  </si>
+  <si>
+    <t>aicte_approved</t>
   </si>
 </sst>
 </file>
@@ -488,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
@@ -497,16 +500,17 @@
     <col min="4" max="4" width="13.44140625" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="12.109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="11" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -538,28 +542,31 @@
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:17" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -594,21 +601,24 @@
         <v>21</v>
       </c>
       <c r="L2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="M2" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="M2" s="2" t="s">
-        <v>22</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>22</v>
       </c>
       <c r="O2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="Q2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="R2" s="2" t="s">
         <v>24</v>
       </c>
     </row>
@@ -676,17 +686,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4330971E-46F0-4063-9D60-3EA0B29B5B12}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>29</v>
       </c>
@@ -697,16 +707,19 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="27.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="27.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>17</v>
       </c>
@@ -717,12 +730,15 @@
         <v>17</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>19</v>
-      </c>
       <c r="F2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>